<commit_message>
Auto-build: public xlsx export (no Notes, no internal dates)
</commit_message>
<xml_diff>
--- a/docs/data/afts-recalls-public.xlsx
+++ b/docs/data/afts-recalls-public.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recalls" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Recalls" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17657,7 +17657,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Generated: 2026-04-29 11:35 UTC</t>
+          <t>Generated: 2026-04-29 20:04 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>